<commit_message>
Get NAV of all the 19 stocks.xlsx
</commit_message>
<xml_diff>
--- a/stocks.xlsx
+++ b/stocks.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bansal_s\PyCharmMiscProject\Day 36\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Suresh\PycharmProjects\scheduled-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D41080E-6A05-46A0-86AB-36BF90A0ADE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71B67D93-8AB1-4050-8C91-2C8C97B6C73C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DBF5B9E9-41A4-47B0-865D-D7F003C09541}"/>
   </bookViews>
@@ -612,7 +612,7 @@
         <v>172.81013157894733</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>42</v>
@@ -631,7 +631,7 @@
         <v>503.69607032558139</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>42</v>
@@ -650,7 +650,7 @@
         <v>57.830406026058633</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>42</v>
@@ -669,7 +669,7 @@
         <v>110.19422105670104</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>42</v>
@@ -688,7 +688,7 @@
         <v>554.99766666666665</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>42</v>
@@ -707,7 +707,7 @@
         <v>167.3698870779221</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>42</v>
@@ -726,7 +726,7 @@
         <v>26.013505000000002</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>42</v>
@@ -764,7 +764,7 @@
         <v>23.33278516426159</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>42</v>
@@ -783,7 +783,7 @@
         <v>177.50579930069932</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>42</v>
@@ -802,7 +802,7 @@
         <v>104.72509670487105</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>42</v>
@@ -821,7 +821,7 @@
         <v>659.84090909090912</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>42</v>
@@ -840,7 +840,7 @@
         <v>119.79999999999998</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>42</v>
@@ -859,7 +859,7 @@
         <v>717.05555555555554</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>42</v>
@@ -878,7 +878,7 @@
         <v>44.493333333333332</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>42</v>
@@ -897,7 +897,7 @@
         <v>193</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>42</v>
@@ -916,7 +916,7 @@
         <v>155.83000000000001</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>42</v>
@@ -935,7 +935,7 @@
         <v>415</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>42</v>
@@ -954,7 +954,7 @@
         <v>2165</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>42</v>

</xml_diff>